<commit_message>
Key states FL LA TX; harmonized elevation, Builty cost and funding, ICC and HMGP on the panel; analysis.dta declutter with diagnostics file; ATTOM value floor upstream; loose Builty-ATTOM address rungs as the standard ladder; master.do paths by user and run order (issues 13, 16, 23-26)
</commit_message>
<xml_diff>
--- a/output/tables/builty_coverage_by_state.xlsx
+++ b/output/tables/builty_coverage_by_state.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="14" uniqueCount="14">
   <si>
     <t>State</t>
   </si>
@@ -22,9 +22,6 @@
   </si>
   <si>
     <t>LA</t>
-  </si>
-  <si>
-    <t>NJ</t>
   </si>
   <si>
     <t>TX</t>
@@ -103,7 +100,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -111,34 +108,34 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>9</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>10</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>12</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>13</v>
-      </c>
-      <c r="K1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2">
@@ -216,22 +213,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="1">
-        <v>21</v>
+        <v>206</v>
       </c>
       <c r="C4" s="1">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="D4" s="1">
-        <v>23.809524536132813</v>
+        <v>17.961164474487305</v>
       </c>
       <c r="E4" s="1">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="F4" s="1">
-        <v>19.047618865966797</v>
+        <v>16.504854202270508</v>
       </c>
       <c r="G4" s="1">
-        <v>3.1619834187709639</v>
+        <v>6.8734253416869189</v>
       </c>
       <c r="H4" s="1">
         <v>1990</v>
@@ -240,44 +237,9 @@
         <v>2026</v>
       </c>
       <c r="J4" s="1">
-        <v>82.853790283203125</v>
+        <v>98.650436401367188</v>
       </c>
       <c r="K4" s="1">
-        <v>49.997097015380859</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1">
-        <v>206</v>
-      </c>
-      <c r="C5" s="1">
-        <v>37</v>
-      </c>
-      <c r="D5" s="1">
-        <v>17.961164474487305</v>
-      </c>
-      <c r="E5" s="1">
-        <v>34</v>
-      </c>
-      <c r="F5" s="1">
-        <v>16.504854202270508</v>
-      </c>
-      <c r="G5" s="1">
-        <v>6.8734253416869189</v>
-      </c>
-      <c r="H5" s="1">
-        <v>1990</v>
-      </c>
-      <c r="I5" s="1">
-        <v>2026</v>
-      </c>
-      <c r="J5" s="1">
-        <v>98.650436401367188</v>
-      </c>
-      <c r="K5" s="1">
         <v>96.919525146484375</v>
       </c>
     </row>

</xml_diff>